<commit_message>
feat: add UI components, database configuration, and templates for QR attendance system
</commit_message>
<xml_diff>
--- a/backend/test_export_october.xlsx
+++ b/backend/test_export_october.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="395" uniqueCount="111">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="384" uniqueCount="110">
   <si>
     <t>School Form 2 (SF2) Daily Attendance Report of Learners</t>
   </si>
@@ -126,9 +126,6 @@
   </si>
   <si>
     <t>HERANI, ANTHONY JR QUINTERO</t>
-  </si>
-  <si>
-    <t>JASTEN C CABATO</t>
   </si>
   <si>
     <t>LAPITAN, GIDEON NATIVIDAD</t>
@@ -2478,7 +2475,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:AU72"/>
+  <dimension ref="A1:AV72"/>
   <sheetFormatPr defaultRowHeight="12.75" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="8.7109375" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="1.5703125" style="1" customWidth="1"/>
@@ -3458,7 +3455,7 @@
       <c r="AT13" s="71"/>
       <c r="AU13" s="69"/>
     </row>
-    <row r="14" ht="20.1" customHeight="1" spans="1:47" x14ac:dyDescent="0.25">
+    <row r="14" ht="20.1" customHeight="1" spans="1:48" x14ac:dyDescent="0.25">
       <c r="A14" s="55">
         <v>7</v>
       </c>
@@ -3476,7 +3473,7 @@
         <v>28</v>
       </c>
       <c r="I14" s="61" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="J14" s="26" t="s">
         <v>28</v>
@@ -3505,7 +3502,7 @@
       </c>
       <c r="W14" s="25"/>
       <c r="X14" s="27" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="Y14" s="25"/>
       <c r="Z14" s="63"/>
@@ -3534,8 +3531,9 @@
       <c r="AS14" s="71"/>
       <c r="AT14" s="71"/>
       <c r="AU14" s="69"/>
+      <c r="AV14" s="1"/>
     </row>
-    <row r="15" ht="20.1" customHeight="1" spans="1:47" x14ac:dyDescent="0.25">
+    <row r="15" ht="20.1" customHeight="1" spans="1:48" x14ac:dyDescent="0.25">
       <c r="A15" s="55">
         <v>8</v>
       </c>
@@ -3559,7 +3557,7 @@
         <v>28</v>
       </c>
       <c r="K15" s="31" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="L15" s="24" t="s">
         <v>28</v>
@@ -3599,11 +3597,11 @@
       <c r="AK15" s="27"/>
       <c r="AL15" s="67"/>
       <c r="AM15" s="68">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="AN15" s="69"/>
       <c r="AO15" s="68">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="AP15" s="69"/>
       <c r="AQ15" s="70"/>
@@ -3611,8 +3609,9 @@
       <c r="AS15" s="71"/>
       <c r="AT15" s="71"/>
       <c r="AU15" s="69"/>
+      <c r="AV15" s="1"/>
     </row>
-    <row r="16" ht="20.1" customHeight="1" spans="1:47" x14ac:dyDescent="0.25">
+    <row r="16" ht="20.1" customHeight="1" spans="1:48" x14ac:dyDescent="0.25">
       <c r="A16" s="55">
         <v>9</v>
       </c>
@@ -3636,7 +3635,7 @@
         <v>28</v>
       </c>
       <c r="K16" s="79" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="L16" s="24" t="s">
         <v>28</v>
@@ -3676,11 +3675,11 @@
       <c r="AK16" s="27"/>
       <c r="AL16" s="67"/>
       <c r="AM16" s="68">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="AN16" s="69"/>
       <c r="AO16" s="68">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AP16" s="69"/>
       <c r="AQ16" s="70"/>
@@ -3688,8 +3687,9 @@
       <c r="AS16" s="71"/>
       <c r="AT16" s="71"/>
       <c r="AU16" s="69"/>
+      <c r="AV16" s="1"/>
     </row>
-    <row r="17" ht="20.1" customHeight="1" spans="1:47" x14ac:dyDescent="0.25">
+    <row r="17" ht="20.1" customHeight="1" spans="1:48" x14ac:dyDescent="0.25">
       <c r="A17" s="55">
         <v>10</v>
       </c>
@@ -3710,7 +3710,7 @@
         <v>28</v>
       </c>
       <c r="J17" s="26" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="K17" s="31" t="s">
         <v>28</v>
@@ -3753,11 +3753,11 @@
       <c r="AK17" s="27"/>
       <c r="AL17" s="67"/>
       <c r="AM17" s="68">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="AN17" s="69"/>
       <c r="AO17" s="68">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="AP17" s="69"/>
       <c r="AQ17" s="70"/>
@@ -3765,8 +3765,9 @@
       <c r="AS17" s="71"/>
       <c r="AT17" s="71"/>
       <c r="AU17" s="69"/>
+      <c r="AV17" s="1"/>
     </row>
-    <row r="18" ht="20.1" customHeight="1" spans="1:47" x14ac:dyDescent="0.25">
+    <row r="18" ht="20.1" customHeight="1" spans="1:48" x14ac:dyDescent="0.25">
       <c r="A18" s="55">
         <v>11</v>
       </c>
@@ -3787,7 +3788,7 @@
         <v>28</v>
       </c>
       <c r="J18" s="61" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="K18" s="31" t="s">
         <v>28</v>
@@ -3830,11 +3831,11 @@
       <c r="AK18" s="27"/>
       <c r="AL18" s="67"/>
       <c r="AM18" s="68">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="AN18" s="69"/>
       <c r="AO18" s="68">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AP18" s="69"/>
       <c r="AQ18" s="70"/>
@@ -3842,8 +3843,9 @@
       <c r="AS18" s="71"/>
       <c r="AT18" s="71"/>
       <c r="AU18" s="69"/>
+      <c r="AV18" s="1"/>
     </row>
-    <row r="19" ht="20.1" customHeight="1" spans="1:47" x14ac:dyDescent="0.25">
+    <row r="19" ht="20.1" customHeight="1" spans="1:48" x14ac:dyDescent="0.25">
       <c r="A19" s="55">
         <v>12</v>
       </c>
@@ -3861,7 +3863,7 @@
         <v>28</v>
       </c>
       <c r="I19" s="26" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="J19" s="26" t="s">
         <v>28</v>
@@ -3907,11 +3909,11 @@
       <c r="AK19" s="27"/>
       <c r="AL19" s="67"/>
       <c r="AM19" s="68">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="AN19" s="69"/>
       <c r="AO19" s="68">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="AP19" s="69"/>
       <c r="AQ19" s="70"/>
@@ -3919,56 +3921,35 @@
       <c r="AS19" s="71"/>
       <c r="AT19" s="71"/>
       <c r="AU19" s="69"/>
+      <c r="AV19" s="1"/>
     </row>
-    <row r="20" ht="20.1" customHeight="1" spans="1:47" x14ac:dyDescent="0.25">
+    <row r="20" ht="20.1" customHeight="1" spans="1:48" x14ac:dyDescent="0.25">
       <c r="A20" s="55">
         <v>13</v>
       </c>
       <c r="B20" s="56"/>
-      <c r="C20" s="59" t="s">
-        <v>43</v>
-      </c>
+      <c r="C20" s="59"/>
       <c r="D20" s="77"/>
       <c r="E20" s="78"/>
-      <c r="F20" s="24" t="s">
-        <v>28</v>
-      </c>
+      <c r="F20" s="24"/>
       <c r="G20" s="25"/>
-      <c r="H20" s="26" t="s">
-        <v>28</v>
-      </c>
-      <c r="I20" s="61" t="s">
-        <v>27</v>
-      </c>
-      <c r="J20" s="26" t="s">
-        <v>28</v>
-      </c>
-      <c r="K20" s="31" t="s">
-        <v>28</v>
-      </c>
-      <c r="L20" s="24" t="s">
-        <v>28</v>
-      </c>
+      <c r="H20" s="26"/>
+      <c r="I20" s="61"/>
+      <c r="J20" s="26"/>
+      <c r="K20" s="31"/>
+      <c r="L20" s="24"/>
       <c r="M20" s="25"/>
       <c r="N20" s="26"/>
-      <c r="O20" s="61" t="s">
-        <v>27</v>
-      </c>
+      <c r="O20" s="61"/>
       <c r="P20" s="26"/>
       <c r="Q20" s="31"/>
-      <c r="R20" s="60" t="s">
-        <v>27</v>
-      </c>
+      <c r="R20" s="60"/>
       <c r="S20" s="25"/>
       <c r="T20" s="26"/>
       <c r="U20" s="26"/>
-      <c r="V20" s="62" t="s">
-        <v>27</v>
-      </c>
+      <c r="V20" s="62"/>
       <c r="W20" s="25"/>
-      <c r="X20" s="62" t="s">
-        <v>27</v>
-      </c>
+      <c r="X20" s="62"/>
       <c r="Y20" s="25"/>
       <c r="Z20" s="63"/>
       <c r="AA20" s="64"/>
@@ -3983,19 +3964,16 @@
       <c r="AJ20" s="26"/>
       <c r="AK20" s="27"/>
       <c r="AL20" s="67"/>
-      <c r="AM20" s="68">
-        <v>5</v>
-      </c>
+      <c r="AM20" s="68"/>
       <c r="AN20" s="69"/>
-      <c r="AO20" s="68">
-        <v>5</v>
-      </c>
+      <c r="AO20" s="68"/>
       <c r="AP20" s="69"/>
       <c r="AQ20" s="70"/>
       <c r="AR20" s="71"/>
       <c r="AS20" s="71"/>
       <c r="AT20" s="71"/>
       <c r="AU20" s="69"/>
+      <c r="AV20" s="1"/>
     </row>
     <row r="21" ht="20.1" customHeight="1" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A21" s="55">
@@ -4152,37 +4130,37 @@
     </row>
     <row r="24" ht="20.1" customHeight="1" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A24" s="83">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B24" s="84"/>
       <c r="C24" s="85" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D24" s="86"/>
       <c r="E24" s="87"/>
       <c r="F24" s="88">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="G24" s="89"/>
       <c r="H24" s="90">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="I24" s="90">
+        <v>10</v>
+      </c>
+      <c r="J24" s="90">
+        <v>10.5</v>
+      </c>
+      <c r="K24" s="91">
+        <v>10.5</v>
+      </c>
+      <c r="L24" s="92">
         <v>11</v>
-      </c>
-      <c r="J24" s="90">
-        <v>11.5</v>
-      </c>
-      <c r="K24" s="91">
-        <v>11.5</v>
-      </c>
-      <c r="L24" s="92">
-        <v>13</v>
       </c>
       <c r="M24" s="89"/>
       <c r="N24" s="90"/>
       <c r="O24" s="90">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P24" s="90"/>
       <c r="Q24" s="91"/>
@@ -4193,11 +4171,11 @@
       <c r="T24" s="90"/>
       <c r="U24" s="90"/>
       <c r="V24" s="92">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="W24" s="89"/>
       <c r="X24" s="92">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Y24" s="93"/>
       <c r="Z24" s="94"/>
@@ -4214,11 +4192,11 @@
       <c r="AK24" s="92"/>
       <c r="AL24" s="97"/>
       <c r="AM24" s="98">
-        <v>55</v>
+        <v>51</v>
       </c>
       <c r="AN24" s="99"/>
       <c r="AO24" s="98">
-        <v>75</v>
+        <v>69</v>
       </c>
       <c r="AP24" s="99"/>
       <c r="AQ24" s="98" t="s">
@@ -4235,7 +4213,7 @@
       </c>
       <c r="B25" s="56"/>
       <c r="C25" s="57" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="D25" s="101"/>
       <c r="E25" s="102"/>
@@ -4312,7 +4290,7 @@
       </c>
       <c r="B26" s="56"/>
       <c r="C26" s="59" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D26" s="77"/>
       <c r="E26" s="78"/>
@@ -4389,7 +4367,7 @@
       </c>
       <c r="B27" s="56"/>
       <c r="C27" s="59" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="D27" s="77"/>
       <c r="E27" s="78"/>
@@ -4466,7 +4444,7 @@
       </c>
       <c r="B28" s="56"/>
       <c r="C28" s="59" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="D28" s="77"/>
       <c r="E28" s="78"/>
@@ -4543,7 +4521,7 @@
       </c>
       <c r="B29" s="56"/>
       <c r="C29" s="59" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="D29" s="77"/>
       <c r="E29" s="78"/>
@@ -4620,7 +4598,7 @@
       </c>
       <c r="B30" s="56"/>
       <c r="C30" s="59" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="D30" s="77"/>
       <c r="E30" s="78"/>
@@ -4697,7 +4675,7 @@
       </c>
       <c r="B31" s="56"/>
       <c r="C31" s="59" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="D31" s="77"/>
       <c r="E31" s="78"/>
@@ -4774,7 +4752,7 @@
       </c>
       <c r="B32" s="56"/>
       <c r="C32" s="59" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D32" s="77"/>
       <c r="E32" s="78"/>
@@ -4851,7 +4829,7 @@
       </c>
       <c r="B33" s="56"/>
       <c r="C33" s="59" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="D33" s="77"/>
       <c r="E33" s="78"/>
@@ -4928,7 +4906,7 @@
       </c>
       <c r="B34" s="56"/>
       <c r="C34" s="59" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="D34" s="77"/>
       <c r="E34" s="78"/>
@@ -5005,7 +4983,7 @@
       </c>
       <c r="B35" s="56"/>
       <c r="C35" s="105" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="D35" s="106"/>
       <c r="E35" s="107"/>
@@ -5082,7 +5060,7 @@
       </c>
       <c r="B36" s="56"/>
       <c r="C36" s="105" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="D36" s="106"/>
       <c r="E36" s="107"/>
@@ -5159,7 +5137,7 @@
       </c>
       <c r="B37" s="56"/>
       <c r="C37" s="105" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="D37" s="106"/>
       <c r="E37" s="107"/>
@@ -5236,7 +5214,7 @@
       </c>
       <c r="B38" s="84"/>
       <c r="C38" s="85" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="D38" s="86"/>
       <c r="E38" s="87"/>
@@ -5311,52 +5289,52 @@
     </row>
     <row r="39" ht="20.1" customHeight="1" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A39" s="83">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B39" s="84"/>
       <c r="C39" s="108" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="D39" s="109"/>
       <c r="E39" s="110"/>
       <c r="F39" s="88">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="G39" s="89"/>
       <c r="H39" s="90">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="I39" s="90">
+        <v>23</v>
+      </c>
+      <c r="J39" s="90">
+        <v>22</v>
+      </c>
+      <c r="K39" s="91">
+        <v>23</v>
+      </c>
+      <c r="L39" s="92">
         <v>24</v>
-      </c>
-      <c r="J39" s="90">
-        <v>23</v>
-      </c>
-      <c r="K39" s="91">
-        <v>24</v>
-      </c>
-      <c r="L39" s="92">
-        <v>26</v>
       </c>
       <c r="M39" s="89"/>
       <c r="N39" s="111"/>
       <c r="O39" s="112">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P39" s="113"/>
       <c r="Q39" s="114"/>
       <c r="R39" s="92">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S39" s="89"/>
       <c r="T39" s="111"/>
       <c r="U39" s="115"/>
       <c r="V39" s="93">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="W39" s="89"/>
       <c r="X39" s="92">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="Y39" s="93"/>
       <c r="Z39" s="116"/>
@@ -5373,11 +5351,11 @@
       <c r="AK39" s="113"/>
       <c r="AL39" s="114"/>
       <c r="AM39" s="98">
-        <v>109</v>
+        <v>105</v>
       </c>
       <c r="AN39" s="99"/>
       <c r="AO39" s="98">
-        <v>151</v>
+        <v>145</v>
       </c>
       <c r="AP39" s="99"/>
       <c r="AQ39" s="98" t="s">
@@ -5390,7 +5368,7 @@
     </row>
     <row r="40" ht="9.95" customHeight="1" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A40" s="118" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B40" s="1"/>
       <c r="C40" s="1"/>
@@ -5417,7 +5395,7 @@
       <c r="X40" s="1"/>
       <c r="Y40" s="5"/>
       <c r="Z40" s="119" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="AA40" s="120"/>
       <c r="AB40" s="121"/>
@@ -5432,16 +5410,16 @@
       <c r="AK40" s="122"/>
       <c r="AL40" s="5"/>
       <c r="AM40" s="123" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="AN40" s="124"/>
       <c r="AO40" s="125"/>
       <c r="AP40" s="123" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="AQ40" s="125"/>
       <c r="AR40" s="126" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="AS40" s="127"/>
       <c r="AT40" s="127"/>
@@ -5449,7 +5427,7 @@
     </row>
     <row r="41" ht="9.95" customHeight="1" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A41" s="129" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B41" s="1"/>
       <c r="C41" s="1"/>
@@ -5476,7 +5454,7 @@
       <c r="X41" s="1"/>
       <c r="Y41" s="5"/>
       <c r="Z41" s="130" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="AA41" s="131"/>
       <c r="AB41" s="131"/>
@@ -5502,7 +5480,7 @@
         <v>19</v>
       </c>
       <c r="AT41" s="137" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="AU41" s="138"/>
     </row>
@@ -5546,7 +5524,7 @@
       <c r="AK42" s="132"/>
       <c r="AL42" s="5"/>
       <c r="AM42" s="139" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="AN42" s="140"/>
       <c r="AO42" s="140"/>
@@ -5590,7 +5568,7 @@
       <c r="X43" s="1"/>
       <c r="Y43" s="5"/>
       <c r="Z43" s="119" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="AA43" s="120"/>
       <c r="AB43" s="120"/>
@@ -5654,12 +5632,12 @@
       <c r="AK44" s="145"/>
       <c r="AL44" s="5"/>
       <c r="AM44" s="153" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="AN44" s="154"/>
       <c r="AO44" s="155"/>
       <c r="AP44" s="156" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="AQ44" s="157"/>
       <c r="AR44" s="142">
@@ -5676,14 +5654,14 @@
     <row r="45" ht="8.1" customHeight="1" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A45" s="5"/>
       <c r="B45" s="140" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C45" s="1"/>
       <c r="D45" s="1"/>
       <c r="E45" s="1"/>
       <c r="F45" s="1"/>
       <c r="G45" s="158" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="H45" s="158"/>
       <c r="I45" s="158"/>
@@ -5698,7 +5676,7 @@
       <c r="R45" s="158"/>
       <c r="S45" s="158"/>
       <c r="T45" s="158" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="U45" s="1"/>
       <c r="V45" s="1"/>
@@ -5706,7 +5684,7 @@
       <c r="X45" s="5"/>
       <c r="Y45" s="5"/>
       <c r="Z45" s="119" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="AA45" s="120"/>
       <c r="AB45" s="120"/>
@@ -5770,7 +5748,7 @@
       <c r="AK46" s="145"/>
       <c r="AL46" s="5"/>
       <c r="AM46" s="163" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="AN46" s="164"/>
       <c r="AO46" s="164"/>
@@ -5789,7 +5767,7 @@
       <c r="E47" s="1"/>
       <c r="F47" s="1"/>
       <c r="G47" s="158" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="H47" s="1"/>
       <c r="I47" s="1"/>
@@ -5810,7 +5788,7 @@
       <c r="X47" s="5"/>
       <c r="Y47" s="5"/>
       <c r="Z47" s="166" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="AA47" s="167"/>
       <c r="AB47" s="167"/>
@@ -5837,14 +5815,14 @@
     <row r="48" ht="9.95" customHeight="1" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A48" s="5"/>
       <c r="B48" s="140" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="C48" s="1"/>
       <c r="D48" s="1"/>
       <c r="E48" s="1"/>
       <c r="F48" s="1"/>
       <c r="G48" s="162" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="H48" s="162"/>
       <c r="I48" s="162"/>
@@ -5878,7 +5856,7 @@
       <c r="AK48" s="168"/>
       <c r="AL48" s="5"/>
       <c r="AM48" s="172" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="AN48" s="173"/>
       <c r="AO48" s="173"/>
@@ -5903,7 +5881,7 @@
       <c r="E49" s="1"/>
       <c r="F49" s="1"/>
       <c r="G49" s="158" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="H49" s="1"/>
       <c r="I49" s="1"/>
@@ -5937,7 +5915,7 @@
       <c r="AK49" s="168"/>
       <c r="AL49" s="5"/>
       <c r="AM49" s="178" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="AN49" s="179"/>
       <c r="AO49" s="179"/>
@@ -5951,14 +5929,14 @@
     <row r="50" ht="9.95" customHeight="1" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A50" s="5"/>
       <c r="B50" s="140" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="C50" s="1"/>
       <c r="D50" s="1"/>
       <c r="E50" s="1"/>
       <c r="F50" s="1"/>
       <c r="G50" s="162" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="H50" s="162"/>
       <c r="I50" s="162"/>
@@ -5973,7 +5951,7 @@
       <c r="R50" s="162"/>
       <c r="S50" s="162"/>
       <c r="T50" s="158" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="U50" s="1"/>
       <c r="V50" s="1"/>
@@ -5994,7 +5972,7 @@
       <c r="AK50" s="168"/>
       <c r="AL50" s="5"/>
       <c r="AM50" s="172" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="AN50" s="173"/>
       <c r="AO50" s="173"/>
@@ -6019,7 +5997,7 @@
       <c r="E51" s="1"/>
       <c r="F51" s="1"/>
       <c r="G51" s="158" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="H51" s="1"/>
       <c r="I51" s="1"/>
@@ -6040,7 +6018,7 @@
       <c r="X51" s="5"/>
       <c r="Y51" s="5"/>
       <c r="Z51" s="119" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="AA51" s="120"/>
       <c r="AB51" s="120"/>
@@ -6055,7 +6033,7 @@
       <c r="AK51" s="145"/>
       <c r="AL51" s="5"/>
       <c r="AM51" s="178" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="AN51" s="179"/>
       <c r="AO51" s="179"/>
@@ -6093,7 +6071,7 @@
       <c r="X52" s="5"/>
       <c r="Y52" s="5"/>
       <c r="Z52" s="166" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="AA52" s="167"/>
       <c r="AB52" s="167"/>
@@ -6108,7 +6086,7 @@
       <c r="AK52" s="168"/>
       <c r="AL52" s="5"/>
       <c r="AM52" s="163" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="AN52" s="164"/>
       <c r="AO52" s="164"/>
@@ -6127,7 +6105,7 @@
     </row>
     <row r="53" ht="5.1" customHeight="1" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A53" s="192" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B53" s="1"/>
       <c r="C53" s="1"/>
@@ -6216,7 +6194,7 @@
       <c r="AK54" s="168"/>
       <c r="AL54" s="5"/>
       <c r="AM54" s="169" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="AN54" s="170"/>
       <c r="AO54" s="170"/>
@@ -6273,7 +6251,7 @@
       <c r="AK55" s="168"/>
       <c r="AL55" s="5"/>
       <c r="AM55" s="169" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="AN55" s="170"/>
       <c r="AO55" s="170"/>
@@ -6330,7 +6308,7 @@
       <c r="AK56" s="168"/>
       <c r="AL56" s="5"/>
       <c r="AM56" s="199" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="AN56" s="200"/>
       <c r="AO56" s="200"/>
@@ -6350,7 +6328,7 @@
     <row r="57" ht="3.95" customHeight="1" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A57" s="5"/>
       <c r="B57" s="202" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="C57" s="203"/>
       <c r="D57" s="203"/>
@@ -6376,7 +6354,7 @@
       <c r="X57" s="204"/>
       <c r="Y57" s="5"/>
       <c r="Z57" s="119" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="AA57" s="120"/>
       <c r="AB57" s="120"/>
@@ -6440,7 +6418,7 @@
       <c r="AK58" s="145"/>
       <c r="AL58" s="5"/>
       <c r="AM58" s="36" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="AN58" s="210"/>
       <c r="AO58" s="210"/>
@@ -6484,7 +6462,7 @@
       <c r="X59" s="209"/>
       <c r="Y59" s="5"/>
       <c r="Z59" s="166" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="AA59" s="167"/>
       <c r="AB59" s="167"/>
@@ -6548,7 +6526,7 @@
       <c r="AK60" s="168"/>
       <c r="AL60" s="5"/>
       <c r="AM60" s="36" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="AN60" s="210"/>
       <c r="AO60" s="210"/>
@@ -6690,7 +6668,7 @@
       <c r="X63" s="5"/>
       <c r="Y63" s="5"/>
       <c r="Z63" s="119" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="AA63" s="120"/>
       <c r="AB63" s="120"/>
@@ -6705,7 +6683,7 @@
       <c r="AK63" s="145"/>
       <c r="AL63" s="5"/>
       <c r="AM63" s="219" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="AN63" s="1"/>
       <c r="AO63" s="1"/>
@@ -6743,7 +6721,7 @@
       <c r="X64" s="5"/>
       <c r="Y64" s="5"/>
       <c r="Z64" s="166" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="AA64" s="167"/>
       <c r="AB64" s="167"/>
@@ -6808,7 +6786,7 @@
       <c r="AL65" s="5"/>
       <c r="AM65" s="5"/>
       <c r="AN65" s="220" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="AO65" s="220"/>
       <c r="AP65" s="220"/>
@@ -6845,7 +6823,7 @@
       <c r="X66" s="5"/>
       <c r="Y66" s="5"/>
       <c r="Z66" s="119" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="AA66" s="120"/>
       <c r="AB66" s="120"/>
@@ -6896,7 +6874,7 @@
       <c r="X67" s="5"/>
       <c r="Y67" s="5"/>
       <c r="Z67" s="166" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="AA67" s="167"/>
       <c r="AB67" s="167"/>
@@ -6912,7 +6890,7 @@
       <c r="AL67" s="5"/>
       <c r="AM67" s="5"/>
       <c r="AN67" s="222" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="AO67" s="1"/>
       <c r="AP67" s="1"/>
@@ -6949,7 +6927,7 @@
       <c r="X68" s="5"/>
       <c r="Y68" s="5"/>
       <c r="Z68" s="223" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="AA68" s="224"/>
       <c r="AB68" s="224"/>
@@ -7013,7 +6991,7 @@
       <c r="AK69" s="228"/>
       <c r="AL69" s="5"/>
       <c r="AM69" s="219" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="AN69" s="1"/>
       <c r="AO69" s="1"/>
@@ -7100,7 +7078,7 @@
       <c r="X71" s="5"/>
       <c r="Y71" s="5"/>
       <c r="Z71" s="221" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="AA71" s="221"/>
       <c r="AB71" s="221"/>
@@ -7116,7 +7094,7 @@
       <c r="AL71" s="5"/>
       <c r="AM71" s="5"/>
       <c r="AN71" s="221" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="AO71" s="221"/>
       <c r="AP71" s="221"/>
@@ -7153,7 +7131,7 @@
       <c r="X72" s="5"/>
       <c r="Y72" s="5"/>
       <c r="Z72" s="229" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="AA72" s="229"/>
       <c r="AB72" s="229"/>
@@ -7169,7 +7147,7 @@
       <c r="AL72" s="5"/>
       <c r="AM72" s="5"/>
       <c r="AN72" s="222" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="AO72" s="1"/>
       <c r="AP72" s="1"/>

</xml_diff>